<commit_message>
Updates to compare_scenario_pj_to_2040 to reflect conditional formatting above 5%
</commit_message>
<xml_diff>
--- a/outputs/pct_of_2040/AggregatedDemand_combined_node_locations_for_energy_conversion_country_constrained_pct_of_2040.xlsx
+++ b/outputs/pct_of_2040/AggregatedDemand_combined_node_locations_for_energy_conversion_country_constrained_pct_of_2040.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="comparison" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="over_5pct_summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,7 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -61,7 +64,7 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -70,8 +73,8 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00FFF2CC"/>
-          <bgColor rgb="00FFF2CC"/>
+          <fgColor rgb="00FCE4D6"/>
+          <bgColor rgb="00FCE4D6"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1397,47 +1400,567 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D2:D14">
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ISO3</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Bau 2040 Low Min Threshold (% of 2040)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Bau 2040 Mid Min Threshold (% of 2040)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Bau 2040 High Min Threshold (% of 2040)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Early Refining 2040 Low Min Threshold (% of 2040)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Early Refining 2040 Mid Min Threshold (% of 2040)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Early Refining 2040 High Min Threshold (% of 2040)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Precursor 2040 Low Min Threshold (% of 2040)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Precursor 2040 Mid Min Threshold (% of 2040)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Precursor 2040 High Min Threshold (% of 2040)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AGO</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>0.0022</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>0.0025</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0.0031</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>0.0255</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>0.0286</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>0.0353</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>0.0132</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>0.0151</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>0.0189</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BDI</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>0.114</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>0.1387</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>0.1712</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0.0819</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>0.09719999999999999</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>0.1191</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>0.0772</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>0.0917</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>0.1117</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BWA</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0.0068</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0.0068</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0.0068</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0.0068</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0.0068</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0.0068</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>0.0068</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>0.0068</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>0.0068</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0.9564</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0.9619</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>0.9696</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>1.014</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>1.0194</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>1.0272</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>0.9592000000000001</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>0.9641</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>0.971</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>KEN</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>0.0001</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>MDG</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0.0738</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>0.07679999999999999</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>0.0808</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>0.08690000000000001</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>0.09089999999999999</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>0.0964</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>0.0866</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>0.0906</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>0.0964</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>MOZ</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>0.008200000000000001</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>0.0119</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>0.0141</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>0.0171</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>0.0127</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>0.0151</v>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>0.0183</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>MWI</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0.0484</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>0.0573</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>0.0692</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>0.057</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>0.0673</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>0.0814</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>0.0605</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>0.0716</v>
+      </c>
+      <c r="J9" s="3" t="n">
+        <v>0.08649999999999999</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>NAM</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>0.005</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TZA</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0.0285</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>0.0343</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>0.0328</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>0.0391</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>0.0477</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>0.0324</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>0.0385</v>
+      </c>
+      <c r="J11" s="3" t="n">
+        <v>0.047</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ZAF</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>0.0038</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>0.0039</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>0.0041</v>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>0.0036</v>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>0.0036</v>
+      </c>
+      <c r="J12" s="3" t="n">
+        <v>0.0038</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ZMB</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0.0323</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>0.0336</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>0.0358</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>0.0595</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>0.0622</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>0.0667</v>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>0.0566</v>
+      </c>
+      <c r="I13" s="3" t="n">
+        <v>0.0587</v>
+      </c>
+      <c r="J13" s="3" t="n">
+        <v>0.0623</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ZWE</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>0.0011</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>0.0012</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>0.0013</v>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>0.0007</v>
+      </c>
+      <c r="J14" s="3" t="n">
+        <v>0.0007</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="B2:B14">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0.05</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F14">
+  <conditionalFormatting sqref="C2:C14">
     <cfRule type="cellIs" priority="2" operator="greaterThan" dxfId="0">
       <formula>0.05</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H14">
+  <conditionalFormatting sqref="D2:D14">
     <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="0">
       <formula>0.05</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J14">
+  <conditionalFormatting sqref="E2:E14">
     <cfRule type="cellIs" priority="4" operator="greaterThan" dxfId="0">
       <formula>0.05</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L2:L14">
+  <conditionalFormatting sqref="F2:F14">
     <cfRule type="cellIs" priority="5" operator="greaterThan" dxfId="0">
       <formula>0.05</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N2:N14">
+  <conditionalFormatting sqref="G2:G14">
     <cfRule type="cellIs" priority="6" operator="greaterThan" dxfId="0">
       <formula>0.05</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P2:P14">
+  <conditionalFormatting sqref="H2:H14">
     <cfRule type="cellIs" priority="7" operator="greaterThan" dxfId="0">
       <formula>0.05</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R2:R14">
+  <conditionalFormatting sqref="I2:I14">
     <cfRule type="cellIs" priority="8" operator="greaterThan" dxfId="0">
       <formula>0.05</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T2:T14">
+  <conditionalFormatting sqref="J2:J14">
     <cfRule type="cellIs" priority="9" operator="greaterThan" dxfId="0">
       <formula>0.05</formula>
     </cfRule>

</xml_diff>